<commit_message>
Sulfate var selection and script updates
</commit_message>
<xml_diff>
--- a/Benchmarks/Water Chemistry/Conductivity/Var selection decisions 1-8-26.xlsx
+++ b/Benchmarks/Water Chemistry/Conductivity/Var selection decisions 1-8-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/sabine_berzins_deq_oregon_gov/Documents/Documents/BioMonORDEQ/Benchmarks/Water Chemistry/Conductivity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{6B8D232A-EEA6-4563-A1A6-87C6EEBA49F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98521123-257F-441E-9E67-17EC12A33FE4}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{6B8D232A-EEA6-4563-A1A6-87C6EEBA49F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9FAE374-0630-4F15-95EF-D1C8C7DC68F3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="1040" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>